<commit_message>
Update: Features, pages, steps and fixtures restructure with new test data
</commit_message>
<xml_diff>
--- a/test-data/Test1.xlsx
+++ b/test-data/Test1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\supri\Pheonix\Phoenix\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{414ADED7-1778-4C0C-AB71-3D47A4EFA00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C158A9B-25B8-431B-925B-71ECEC94F1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8130" yWindow="4680" windowWidth="18000" windowHeight="9540" xr2:uid="{F7E53592-F92F-4807-91B6-69E42A286F67}"/>
+    <workbookView xWindow="2865" yWindow="2760" windowWidth="18000" windowHeight="9540" xr2:uid="{F7E53592-F92F-4807-91B6-69E42A286F67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>PUBLISH DATE</t>
   </si>
@@ -50,7 +50,10 @@
     <t>DOCUMENT NAME</t>
   </si>
   <si>
-    <t>Test1</t>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>DEF</t>
   </si>
 </sst>
 </file>
@@ -423,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CB928A-ACFE-487D-8D27-88888A74B9C7}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -452,6 +455,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46260</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: resolve CreateDocument OverviewTab() async/Promise issue
- Remove async keyword from OverviewTab() method as it doesn't perform async operations
- Fixes error: 'toBeVisible can be only used with Locator object, was called with Promise'
- Test 'User lands on the create document page' now passes successfully
- Refactored CreateDocument page object and step definitions for better locator handling

Fixed Promise/Locator incompatibility in CreateDocument page object. The OverviewTab() method was unnecessarily async, causing it to return a Promise instead of a Locator when called in test steps.
</commit_message>
<xml_diff>
--- a/test-data/Test1.xlsx
+++ b/test-data/Test1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\supri\Pheonix\Phoenix\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{414ADED7-1778-4C0C-AB71-3D47A4EFA00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C158A9B-25B8-431B-925B-71ECEC94F1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8130" yWindow="4680" windowWidth="18000" windowHeight="9540" xr2:uid="{F7E53592-F92F-4807-91B6-69E42A286F67}"/>
+    <workbookView xWindow="2865" yWindow="2760" windowWidth="18000" windowHeight="9540" xr2:uid="{F7E53592-F92F-4807-91B6-69E42A286F67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>PUBLISH DATE</t>
   </si>
@@ -50,7 +50,10 @@
     <t>DOCUMENT NAME</t>
   </si>
   <si>
-    <t>Test1</t>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>DEF</t>
   </si>
 </sst>
 </file>
@@ -423,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CB928A-ACFE-487D-8D27-88888A74B9C7}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -452,6 +455,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46260</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>